<commit_message>
Import 23 Pisa questionnaires with reversed 0-2 scale into shared workbook
</commit_message>
<xml_diff>
--- a/data/ern2026/questionari.xlsx
+++ b/data/ern2026/questionari.xlsx
@@ -164,8 +164,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DatiHEPscape" displayName="DatiHEPscape" ref="A6:N213" headerRowCount="1">
-  <autoFilter ref="A6:N213"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DatiHEPscape" displayName="DatiHEPscape" ref="A6:N236" headerRowCount="1">
+  <autoFilter ref="A6:N236"/>
   <tableColumns count="14">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Q1"/>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OriginaliHEPscape" displayName="OriginaliHEPscape" ref="A1:R208" headerRowCount="1">
-  <autoFilter ref="A1:R208"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OriginaliHEPscape" displayName="OriginaliHEPscape" ref="A1:R231" headerRowCount="1">
+  <autoFilter ref="A1:R231"/>
   <tableColumns count="18">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Q1"/>
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N213"/>
+  <dimension ref="A1:N236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HEPscape! | Evento ERNEST - ERN 2026 | 207 questionari</t>
+          <t>HEPscape! | Evento ERNEST - ERN 2026 | 230 questionari</t>
         </is>
       </c>
     </row>
@@ -11451,44 +11451,1216 @@
         </is>
       </c>
     </row>
+    <row r="214" ht="34" customHeight="1">
+      <c r="A214" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-001</t>
+        </is>
+      </c>
+      <c r="B214" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C214" s="1" t="inlineStr">
+        <is>
+          <t>SIMPATICA</t>
+        </is>
+      </c>
+      <c r="D214" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E214" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F214" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G214" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H214" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I214" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J214" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K214" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="L214" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M214" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N214" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="34" customHeight="1">
+      <c r="A215" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-002</t>
+        </is>
+      </c>
+      <c r="B215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C215" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G215" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K215" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L215" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M215" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N215" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="34" customHeight="1">
+      <c r="A216" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-003</t>
+        </is>
+      </c>
+      <c r="B216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C216" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K216" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L216" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M216" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N216" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="34" customHeight="1">
+      <c r="A217" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-004</t>
+        </is>
+      </c>
+      <c r="B217" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C217" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D217" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E217" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F217" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G217" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="H217" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="I217" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J217" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K217" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L217" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M217" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N217" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="34" customHeight="1">
+      <c r="A218" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-005</t>
+        </is>
+      </c>
+      <c r="B218" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C218" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D218" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E218" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F218" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G218" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H218" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I218" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J218" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K218" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L218" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M218" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N218" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="34" customHeight="1">
+      <c r="A219" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-006</t>
+        </is>
+      </c>
+      <c r="B219" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C219" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D219" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E219" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F219" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G219" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H219" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I219" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J219" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K219" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L219" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M219" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N219" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="34" customHeight="1">
+      <c r="A220" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-007</t>
+        </is>
+      </c>
+      <c r="B220" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C220" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D220" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E220" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F220" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G220" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H220" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I220" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J220" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K220" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L220" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M220" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N220" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="34" customHeight="1">
+      <c r="A221" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-008</t>
+        </is>
+      </c>
+      <c r="B221" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C221" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D221" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E221" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F221" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G221" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H221" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I221" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J221" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K221" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L221" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M221" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N221" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="34" customHeight="1">
+      <c r="A222" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-009</t>
+        </is>
+      </c>
+      <c r="B222" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C222" s="1" t="inlineStr">
+        <is>
+          <t>MI SONO DIVERTITO</t>
+        </is>
+      </c>
+      <c r="D222" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E222" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F222" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G222" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H222" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I222" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J222" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K222" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L222" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M222" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N222" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="34" customHeight="1">
+      <c r="A223" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-010</t>
+        </is>
+      </c>
+      <c r="B223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C223" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H223" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J223" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L223" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M223" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N223" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="34" customHeight="1">
+      <c r="A224" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-011</t>
+        </is>
+      </c>
+      <c r="B224" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C224" s="1" t="inlineStr">
+        <is>
+          <t>INGRESSI BELLO?</t>
+        </is>
+      </c>
+      <c r="D224" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E224" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F224" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G224" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H224" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I224" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J224" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K224" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L224" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M224" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N224" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="34" customHeight="1">
+      <c r="A225" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-012</t>
+        </is>
+      </c>
+      <c r="B225" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C225" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D225" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E225" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F225" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G225" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H225" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I225" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J225" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K225" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L225" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M225" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N225" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="34" customHeight="1">
+      <c r="A226" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-013</t>
+        </is>
+      </c>
+      <c r="B226" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C226" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D226" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E226" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F226" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G226" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H226" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I226" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J226" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K226" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L226" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M226" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N226" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="34" customHeight="1">
+      <c r="A227" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-014</t>
+        </is>
+      </c>
+      <c r="B227" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C227" s="1" t="inlineStr">
+        <is>
+          <t>MOLTO BELLA</t>
+        </is>
+      </c>
+      <c r="D227" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E227" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F227" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G227" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H227" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I227" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J227" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="K227" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L227" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M227" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N227" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="34" customHeight="1">
+      <c r="A228" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-015</t>
+        </is>
+      </c>
+      <c r="B228" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C228" s="1" t="inlineStr">
+        <is>
+          <t>INTERESSANTE</t>
+        </is>
+      </c>
+      <c r="D228" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E228" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F228" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G228" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H228" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I228" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J228" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K228" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L228" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M228" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N228" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="34" customHeight="1">
+      <c r="A229" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-016</t>
+        </is>
+      </c>
+      <c r="B229" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C229" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D229" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E229" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F229" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G229" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H229" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I229" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J229" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K229" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L229" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M229" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N229" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="36" customHeight="1">
+      <c r="A230" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-017</t>
+        </is>
+      </c>
+      <c r="B230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C230" s="1" t="inlineStr">
+        <is>
+          <t>MI E' PIACIUTA TANTISSIMO BELLISSIMA ESPERIENZA</t>
+        </is>
+      </c>
+      <c r="D230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K230" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L230" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M230" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N230" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="34" customHeight="1">
+      <c r="A231" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-018</t>
+        </is>
+      </c>
+      <c r="B231" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C231" s="1" t="inlineStr">
+        <is>
+          <t>CARINA E BEN ORGANIZZATA</t>
+        </is>
+      </c>
+      <c r="D231" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E231" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F231" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G231" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I231" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J231" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K231" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L231" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M231" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N231" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="34" customHeight="1">
+      <c r="A232" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-019</t>
+        </is>
+      </c>
+      <c r="B232" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C232" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="D232" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E232" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F232" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G232" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I232" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K232" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L232" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M232" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N232" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="34" customHeight="1">
+      <c r="A233" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-020</t>
+        </is>
+      </c>
+      <c r="B233" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C233" s="1" t="inlineStr">
+        <is>
+          <t>CARINA E BEN ORGANIZZATA</t>
+        </is>
+      </c>
+      <c r="D233" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E233" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F233" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G233" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I233" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J233" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L233" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M233" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N233" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="34" customHeight="1">
+      <c r="A234" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-021</t>
+        </is>
+      </c>
+      <c r="B234" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C234" s="1" t="inlineStr">
+        <is>
+          <t>INTERESSANTE SCIENTIFICO</t>
+        </is>
+      </c>
+      <c r="D234" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E234" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F234" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G234" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I234" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K234" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L234" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M234" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N234" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="34" customHeight="1">
+      <c r="A235" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-022</t>
+        </is>
+      </c>
+      <c r="B235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C235" s="1" t="inlineStr">
+        <is>
+          <t>BUFFA</t>
+        </is>
+      </c>
+      <c r="D235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G235" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H235" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K235" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M235" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N235" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="34" customHeight="1">
+      <c r="A236" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-023</t>
+        </is>
+      </c>
+      <c r="B236" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C236" s="1" t="inlineStr">
+        <is>
+          <t>BELLO</t>
+        </is>
+      </c>
+      <c r="D236" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E236" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F236" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G236" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="H236" s="1" t="n">
+        <v>999</v>
+      </c>
+      <c r="I236" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K236" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L236" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M236" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="N236" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:L213">
+  <conditionalFormatting sqref="B7:L236">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>999</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="10">
-    <dataValidation sqref="B7:B213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="B7:B236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="D7:D213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="D7:D236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="E7:E213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="E7:E236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="F7:F213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="F7:F236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="G7:G213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="G7:G236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="H7:H213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="H7:H236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="I7:I213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="I7:I236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="J7:J213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="J7:J236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,3,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="K7:K213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="K7:K236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,2,3,4,5,6,7,999"</formula1>
     </dataValidation>
-    <dataValidation sqref="L7:L213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
+    <dataValidation sqref="L7:L236" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Codice non valido" error="Usare i codici in legenda; 999 solo per una risposta vuota." type="list">
       <formula1>"0,1,999"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11505,7 +12677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R208"/>
+  <dimension ref="A1:R231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -28730,6 +29902,1965 @@
       </c>
       <c r="R208" s="1" t="inlineStr"/>
     </row>
+    <row r="209" ht="52" customHeight="1">
+      <c r="A209" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-001</t>
+        </is>
+      </c>
+      <c r="B209" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C209" s="1" t="inlineStr">
+        <is>
+          <t>Simpatica</t>
+        </is>
+      </c>
+      <c r="D209" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E209" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F209" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G209" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H209" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I209" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J209" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K209" s="1" t="inlineStr"/>
+      <c r="L209" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M209" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N209" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=1</t>
+        </is>
+      </c>
+      <c r="O209" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P209" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q209" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R209" s="1" t="inlineStr"/>
+    </row>
+    <row r="210" ht="52" customHeight="1">
+      <c r="A210" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-002</t>
+        </is>
+      </c>
+      <c r="B210" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C210" s="1" t="inlineStr"/>
+      <c r="D210" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E210" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F210" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G210" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H210" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I210" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J210" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K210" s="1" t="inlineStr">
+        <is>
+          <t>11-14</t>
+        </is>
+      </c>
+      <c r="L210" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M210" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N210" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=2</t>
+        </is>
+      </c>
+      <c r="O210" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P210" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q210" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R210" s="1" t="inlineStr"/>
+    </row>
+    <row r="211" ht="52" customHeight="1">
+      <c r="A211" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-003</t>
+        </is>
+      </c>
+      <c r="B211" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C211" s="1" t="inlineStr"/>
+      <c r="D211" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E211" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F211" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G211" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H211" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I211" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J211" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K211" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L211" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M211" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N211" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=3</t>
+        </is>
+      </c>
+      <c r="O211" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P211" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q211" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R211" s="1" t="inlineStr"/>
+    </row>
+    <row r="212" ht="52" customHeight="1">
+      <c r="A212" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-004</t>
+        </is>
+      </c>
+      <c r="B212" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C212" s="1" t="inlineStr"/>
+      <c r="D212" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E212" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F212" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G212" s="1" t="inlineStr"/>
+      <c r="H212" s="1" t="inlineStr"/>
+      <c r="I212" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J212" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K212" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L212" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M212" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N212" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=4</t>
+        </is>
+      </c>
+      <c r="O212" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P212" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q212" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R212" s="1" t="inlineStr"/>
+    </row>
+    <row r="213" ht="52" customHeight="1">
+      <c r="A213" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-005</t>
+        </is>
+      </c>
+      <c r="B213" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C213" s="1" t="inlineStr"/>
+      <c r="D213" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E213" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F213" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G213" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H213" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I213" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J213" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K213" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L213" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M213" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N213" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=5</t>
+        </is>
+      </c>
+      <c r="O213" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P213" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q213" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R213" s="1" t="inlineStr"/>
+    </row>
+    <row r="214" ht="52" customHeight="1">
+      <c r="A214" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-006</t>
+        </is>
+      </c>
+      <c r="B214" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C214" s="1" t="inlineStr"/>
+      <c r="D214" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E214" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F214" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G214" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H214" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I214" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J214" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K214" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L214" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M214" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N214" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=6</t>
+        </is>
+      </c>
+      <c r="O214" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P214" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q214" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R214" s="1" t="inlineStr"/>
+    </row>
+    <row r="215" ht="52" customHeight="1">
+      <c r="A215" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-007</t>
+        </is>
+      </c>
+      <c r="B215" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C215" s="1" t="inlineStr"/>
+      <c r="D215" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E215" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F215" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G215" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H215" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I215" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J215" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K215" s="1" t="inlineStr">
+        <is>
+          <t>11-14</t>
+        </is>
+      </c>
+      <c r="L215" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M215" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N215" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=7</t>
+        </is>
+      </c>
+      <c r="O215" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P215" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q215" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R215" s="1" t="inlineStr"/>
+    </row>
+    <row r="216" ht="52" customHeight="1">
+      <c r="A216" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-008</t>
+        </is>
+      </c>
+      <c r="B216" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C216" s="1" t="inlineStr"/>
+      <c r="D216" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E216" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F216" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G216" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H216" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I216" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J216" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K216" s="1" t="inlineStr">
+        <is>
+          <t>11-14</t>
+        </is>
+      </c>
+      <c r="L216" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M216" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N216" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=8</t>
+        </is>
+      </c>
+      <c r="O216" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P216" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q216" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R216" s="1" t="inlineStr"/>
+    </row>
+    <row r="217" ht="52" customHeight="1">
+      <c r="A217" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-009</t>
+        </is>
+      </c>
+      <c r="B217" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C217" s="1" t="inlineStr">
+        <is>
+          <t>mi sono divertito</t>
+        </is>
+      </c>
+      <c r="D217" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E217" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F217" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G217" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H217" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I217" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J217" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K217" s="1" t="inlineStr">
+        <is>
+          <t>11-14</t>
+        </is>
+      </c>
+      <c r="L217" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M217" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N217" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=9</t>
+        </is>
+      </c>
+      <c r="O217" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P217" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q217" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R217" s="1" t="inlineStr"/>
+    </row>
+    <row r="218" ht="52" customHeight="1">
+      <c r="A218" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-010</t>
+        </is>
+      </c>
+      <c r="B218" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C218" s="1" t="inlineStr"/>
+      <c r="D218" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E218" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F218" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G218" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H218" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I218" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J218" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K218" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L218" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M218" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N218" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=10</t>
+        </is>
+      </c>
+      <c r="O218" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P218" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q218" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R218" s="1" t="inlineStr"/>
+    </row>
+    <row r="219" ht="84" customHeight="1">
+      <c r="A219" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-011</t>
+        </is>
+      </c>
+      <c r="B219" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C219" s="1" t="inlineStr">
+        <is>
+          <t>ingressi bello?</t>
+        </is>
+      </c>
+      <c r="D219" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E219" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F219" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G219" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H219" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I219" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J219" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K219" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L219" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M219" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.
+Q2: Trascrizione fornita dall’utente: punto interrogativo conservato; nessuna verifica su fotografia.</t>
+        </is>
+      </c>
+      <c r="N219" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=11</t>
+        </is>
+      </c>
+      <c r="O219" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P219" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q219" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R219" s="1" t="inlineStr"/>
+    </row>
+    <row r="220" ht="52" customHeight="1">
+      <c r="A220" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-012</t>
+        </is>
+      </c>
+      <c r="B220" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C220" s="1" t="inlineStr"/>
+      <c r="D220" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E220" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F220" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G220" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H220" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I220" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J220" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K220" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L220" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M220" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N220" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=12</t>
+        </is>
+      </c>
+      <c r="O220" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P220" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q220" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R220" s="1" t="inlineStr"/>
+    </row>
+    <row r="221" ht="52" customHeight="1">
+      <c r="A221" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-013</t>
+        </is>
+      </c>
+      <c r="B221" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C221" s="1" t="inlineStr"/>
+      <c r="D221" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E221" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F221" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G221" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H221" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I221" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J221" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K221" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L221" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M221" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N221" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=13</t>
+        </is>
+      </c>
+      <c r="O221" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P221" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q221" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R221" s="1" t="inlineStr"/>
+    </row>
+    <row r="222" ht="52" customHeight="1">
+      <c r="A222" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-014</t>
+        </is>
+      </c>
+      <c r="B222" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C222" s="1" t="inlineStr">
+        <is>
+          <t>molto bella</t>
+        </is>
+      </c>
+      <c r="D222" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E222" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F222" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G222" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H222" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I222" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J222" s="1" t="inlineStr">
+        <is>
+          <t>non risp</t>
+        </is>
+      </c>
+      <c r="K222" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L222" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M222" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N222" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=14</t>
+        </is>
+      </c>
+      <c r="O222" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P222" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q222" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R222" s="1" t="inlineStr"/>
+    </row>
+    <row r="223" ht="52" customHeight="1">
+      <c r="A223" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-015</t>
+        </is>
+      </c>
+      <c r="B223" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C223" s="1" t="inlineStr">
+        <is>
+          <t>interessante</t>
+        </is>
+      </c>
+      <c r="D223" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E223" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F223" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G223" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H223" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I223" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J223" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K223" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L223" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M223" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N223" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=15</t>
+        </is>
+      </c>
+      <c r="O223" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P223" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q223" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R223" s="1" t="inlineStr"/>
+    </row>
+    <row r="224" ht="52" customHeight="1">
+      <c r="A224" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-016</t>
+        </is>
+      </c>
+      <c r="B224" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C224" s="1" t="inlineStr"/>
+      <c r="D224" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E224" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F224" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G224" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H224" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I224" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J224" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K224" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L224" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M224" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N224" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=16</t>
+        </is>
+      </c>
+      <c r="O224" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P224" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q224" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R224" s="1" t="inlineStr"/>
+    </row>
+    <row r="225" ht="52" customHeight="1">
+      <c r="A225" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-017</t>
+        </is>
+      </c>
+      <c r="B225" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C225" s="1" t="inlineStr">
+        <is>
+          <t>mi e' piaciuta tantissimo bellissima esperienza</t>
+        </is>
+      </c>
+      <c r="D225" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E225" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F225" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G225" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H225" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I225" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J225" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K225" s="1" t="inlineStr">
+        <is>
+          <t>11-14</t>
+        </is>
+      </c>
+      <c r="L225" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M225" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N225" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=17</t>
+        </is>
+      </c>
+      <c r="O225" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P225" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q225" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R225" s="1" t="inlineStr"/>
+    </row>
+    <row r="226" ht="84" customHeight="1">
+      <c r="A226" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-018</t>
+        </is>
+      </c>
+      <c r="B226" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C226" s="1" t="inlineStr">
+        <is>
+          <t>carina e ben organizzata</t>
+        </is>
+      </c>
+      <c r="D226" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E226" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F226" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G226" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H226" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I226" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J226" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K226" s="1" t="inlineStr">
+        <is>
+          <t>19-25</t>
+        </is>
+      </c>
+      <c r="L226" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M226" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.
+riga: Le righe 18 e 20 della tabella sono identiche; mantenute come due schede distinte.</t>
+        </is>
+      </c>
+      <c r="N226" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=18</t>
+        </is>
+      </c>
+      <c r="O226" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P226" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q226" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R226" s="1" t="inlineStr"/>
+    </row>
+    <row r="227" ht="52" customHeight="1">
+      <c r="A227" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-019</t>
+        </is>
+      </c>
+      <c r="B227" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C227" s="1" t="inlineStr"/>
+      <c r="D227" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E227" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F227" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G227" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H227" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I227" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J227" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K227" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L227" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M227" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N227" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=19</t>
+        </is>
+      </c>
+      <c r="O227" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P227" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q227" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R227" s="1" t="inlineStr"/>
+    </row>
+    <row r="228" ht="84" customHeight="1">
+      <c r="A228" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-020</t>
+        </is>
+      </c>
+      <c r="B228" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C228" s="1" t="inlineStr">
+        <is>
+          <t>carina e ben organizzata</t>
+        </is>
+      </c>
+      <c r="D228" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E228" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F228" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G228" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H228" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I228" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J228" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K228" s="1" t="inlineStr">
+        <is>
+          <t>19-25</t>
+        </is>
+      </c>
+      <c r="L228" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M228" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.
+riga: Le righe 18 e 20 della tabella sono identiche; mantenute come due schede distinte.</t>
+        </is>
+      </c>
+      <c r="N228" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=20</t>
+        </is>
+      </c>
+      <c r="O228" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P228" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q228" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R228" s="1" t="inlineStr"/>
+    </row>
+    <row r="229" ht="52" customHeight="1">
+      <c r="A229" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-021</t>
+        </is>
+      </c>
+      <c r="B229" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C229" s="1" t="inlineStr">
+        <is>
+          <t>interessante scientifico</t>
+        </is>
+      </c>
+      <c r="D229" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E229" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F229" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G229" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H229" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I229" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J229" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K229" s="1" t="inlineStr">
+        <is>
+          <t>11-14</t>
+        </is>
+      </c>
+      <c r="L229" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M229" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N229" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=21</t>
+        </is>
+      </c>
+      <c r="O229" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P229" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q229" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R229" s="1" t="inlineStr"/>
+    </row>
+    <row r="230" ht="52" customHeight="1">
+      <c r="A230" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-022</t>
+        </is>
+      </c>
+      <c r="B230" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C230" s="1" t="inlineStr">
+        <is>
+          <t>buffa</t>
+        </is>
+      </c>
+      <c r="D230" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E230" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F230" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G230" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H230" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I230" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J230" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K230" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L230" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M230" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N230" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=22</t>
+        </is>
+      </c>
+      <c r="O230" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P230" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q230" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R230" s="1" t="inlineStr"/>
+    </row>
+    <row r="231" ht="52" customHeight="1">
+      <c r="A231" s="1" t="inlineStr">
+        <is>
+          <t>PISA-ERN2026-023</t>
+        </is>
+      </c>
+      <c r="B231" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C231" s="1" t="inlineStr">
+        <is>
+          <t>bello</t>
+        </is>
+      </c>
+      <c r="D231" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E231" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F231" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G231" s="1" t="inlineStr"/>
+      <c r="H231" s="1" t="inlineStr"/>
+      <c r="I231" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J231" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K231" s="1" t="inlineStr">
+        <is>
+          <t>Meno di 11</t>
+        </is>
+      </c>
+      <c r="L231" s="1" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M231" s="1" t="inlineStr">
+        <is>
+          <t>codifica: Valori originali numerici Q1/Q3–Q7 nella scala Pisa: 2→0, 1→1, 0→2. Sì→1, No→0. Celle vuote→999 in Excel.</t>
+        </is>
+      </c>
+      <c r="N231" s="1" t="inlineStr">
+        <is>
+          <t>pisa_tabella_originale.csv#N=23</t>
+        </is>
+      </c>
+      <c r="O231" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="P231" s="1" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="Q231" s="1" t="inlineStr">
+        <is>
+          <t>Confermata</t>
+        </is>
+      </c>
+      <c r="R231" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>